<commit_message>
agent: auto-ship "balance/LIFE-\320\261\320\260\320\273\320\260\320\275\321\201.xlsx", css/style.css, js/app.js, js/content/help.js (+14)
</commit_message>
<xml_diff>
--- a/balance/LIFE-баланс.xlsx
+++ b/balance/LIFE-баланс.xlsx
@@ -30,12 +30,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3696" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3682" uniqueCount="835">
   <si>
     <t>ЖИЗНЬ — таблица баланса</t>
   </si>
   <si>
-    <t>Версия выгрузки: Альфа 0.16.0</t>
+    <t>Версия выгрузки: Альфа 0.17.0</t>
   </si>
   <si>
     <t>Дата: 2026-08-20</t>
@@ -2099,7 +2099,7 @@
     <t>цепочка</t>
   </si>
   <si>
-    <t>Столько циклов подряд с зайцами = устойчивая цепочка (открывает медведя и эру).</t>
+    <t>Столько циклов подряд с зайцами = устойчивая цепочка (открывает медведя и потолок ⚡).</t>
   </si>
   <si>
     <t>arcade.arcadeEnd.noAnimalRenewalGens</t>
@@ -2118,15 +2118,6 @@
   </si>
   <si>
     <t>Раз в столько циклов начисляются очки survival при живой пирамиде.</t>
-  </si>
-  <si>
-    <t>arcade.arcadeEnd.eraAfterChain</t>
-  </si>
-  <si>
-    <t>длина эры</t>
-  </si>
-  <si>
-    <t>После устойчивой цепочки ещё столько циклов — и раунд кончается победой. 0 = бесконечная ферма.</t>
   </si>
   <si>
     <t>arcade.roulette.interval</t>
@@ -3408,57 +3399,57 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>812</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>813</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>814</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>815</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>816</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>817</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>818</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>819</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>820</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>821</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>822</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>823</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>824</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>825</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>826</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>827</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>828</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>3</v>
@@ -3508,7 +3499,7 @@
     </row>
     <row r="3" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>57</v>
@@ -3558,7 +3549,7 @@
     </row>
     <row r="4" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>60</v>
@@ -3608,7 +3599,7 @@
     </row>
     <row r="5" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>63</v>
@@ -3658,7 +3649,7 @@
     </row>
     <row r="6" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>426</v>
@@ -3708,7 +3699,7 @@
     </row>
     <row r="7" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>430</v>
@@ -3758,7 +3749,7 @@
     </row>
     <row r="8" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>433</v>
@@ -3808,7 +3799,7 @@
     </row>
     <row r="9" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>436</v>
@@ -3858,7 +3849,7 @@
     </row>
     <row r="10" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>421</v>
@@ -6304,7 +6295,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -6525,34 +6516,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>696</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>697</v>
-      </c>
-      <c r="C9" s="8">
-        <v>300</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>698</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>677</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6604,10 +6569,10 @@
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C2" s="8">
         <v>100</v>
@@ -6619,10 +6584,10 @@
         <v>246</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>55</v>
@@ -6630,10 +6595,10 @@
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C3" s="8">
         <v>30</v>
@@ -6645,10 +6610,10 @@
         <v>3</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>55</v>
@@ -6656,10 +6621,10 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="C4" s="8">
         <v>30</v>
@@ -6671,10 +6636,10 @@
         <v>3</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>55</v>
@@ -6682,10 +6647,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="C5" s="8">
         <v>25</v>
@@ -6697,10 +6662,10 @@
         <v>3</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>55</v>
@@ -6708,10 +6673,10 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="C6" s="8">
         <v>15</v>
@@ -6723,10 +6688,10 @@
         <v>3</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>55</v>
@@ -6734,10 +6699,10 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="C7" s="8">
         <v>0.1</v>
@@ -6749,10 +6714,10 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>55</v>
@@ -6760,10 +6725,10 @@
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="C8" s="8">
         <v>0.3</v>
@@ -6775,10 +6740,10 @@
         <v>3</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>55</v>
@@ -6786,10 +6751,10 @@
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="C9" s="8">
         <v>0.1</v>
@@ -6801,10 +6766,10 @@
         <v>3</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>55</v>
@@ -6812,10 +6777,10 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="C10" s="8">
         <v>0.5</v>
@@ -6827,10 +6792,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>55</v>
@@ -6838,10 +6803,10 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="C11" s="8">
         <v>0.1</v>
@@ -6853,10 +6818,10 @@
         <v>3</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>55</v>
@@ -6864,10 +6829,10 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="C12" s="8">
         <v>0.3</v>
@@ -6879,10 +6844,10 @@
         <v>3</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>55</v>
@@ -6890,10 +6855,10 @@
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="C13" s="8">
         <v>0.5</v>
@@ -6905,10 +6870,10 @@
         <v>3</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>55</v>
@@ -6916,10 +6881,10 @@
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="C14" s="8">
         <v>1</v>
@@ -6931,10 +6896,10 @@
         <v>3</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>55</v>
@@ -6942,10 +6907,10 @@
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="C15" s="8">
         <v>0.0015</v>
@@ -6957,10 +6922,10 @@
         <v>3</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>55</v>
@@ -6968,10 +6933,10 @@
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="C16" s="8">
         <v>1.8</v>
@@ -6983,10 +6948,10 @@
         <v>3</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>55</v>
@@ -6994,10 +6959,10 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="C17" s="8">
         <v>45</v>
@@ -7009,10 +6974,10 @@
         <v>3</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>55</v>
@@ -7020,10 +6985,10 @@
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="C18" s="8">
         <v>28</v>
@@ -7035,10 +7000,10 @@
         <v>3</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>55</v>
@@ -7155,7 +7120,7 @@
         <v>45</v>
       </c>
       <c r="C4" s="7">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>42</v>
@@ -7211,7 +7176,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
-  <dimension ref="A1:H277"/>
+  <dimension ref="A1:H276"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -7310,7 +7275,7 @@
         <v>45</v>
       </c>
       <c r="C4" s="7">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>42</v>
@@ -13186,7 +13151,7 @@
         <v>697</v>
       </c>
       <c r="C230" s="8">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D230" s="5" t="s">
         <v>42</v>
@@ -13198,7 +13163,7 @@
         <v>698</v>
       </c>
       <c r="G230" s="5" t="s">
-        <v>677</v>
+        <v>699</v>
       </c>
       <c r="H230" s="5" t="s">
         <v>55</v>
@@ -13206,25 +13171,25 @@
     </row>
     <row r="231" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="B231" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="C231" s="8">
+        <v>30</v>
+      </c>
+      <c r="D231" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E231" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F231" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="G231" s="5" t="s">
         <v>699</v>
-      </c>
-      <c r="B231" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="C231" s="8">
-        <v>100</v>
-      </c>
-      <c r="D231" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E231" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="F231" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="G231" s="5" t="s">
-        <v>702</v>
       </c>
       <c r="H231" s="5" t="s">
         <v>55</v>
@@ -13250,7 +13215,7 @@
         <v>705</v>
       </c>
       <c r="G232" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H232" s="5" t="s">
         <v>55</v>
@@ -13264,7 +13229,7 @@
         <v>707</v>
       </c>
       <c r="C233" s="8">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>42</v>
@@ -13276,7 +13241,7 @@
         <v>708</v>
       </c>
       <c r="G233" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H233" s="5" t="s">
         <v>55</v>
@@ -13290,7 +13255,7 @@
         <v>710</v>
       </c>
       <c r="C234" s="8">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D234" s="5" t="s">
         <v>42</v>
@@ -13302,7 +13267,7 @@
         <v>711</v>
       </c>
       <c r="G234" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H234" s="5" t="s">
         <v>55</v>
@@ -13316,7 +13281,7 @@
         <v>713</v>
       </c>
       <c r="C235" s="8">
-        <v>15</v>
+        <v>0.1</v>
       </c>
       <c r="D235" s="5" t="s">
         <v>42</v>
@@ -13328,7 +13293,7 @@
         <v>714</v>
       </c>
       <c r="G235" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H235" s="5" t="s">
         <v>55</v>
@@ -13342,7 +13307,7 @@
         <v>716</v>
       </c>
       <c r="C236" s="8">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D236" s="5" t="s">
         <v>42</v>
@@ -13354,7 +13319,7 @@
         <v>717</v>
       </c>
       <c r="G236" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H236" s="5" t="s">
         <v>55</v>
@@ -13368,7 +13333,7 @@
         <v>719</v>
       </c>
       <c r="C237" s="8">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D237" s="5" t="s">
         <v>42</v>
@@ -13380,7 +13345,7 @@
         <v>720</v>
       </c>
       <c r="G237" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H237" s="5" t="s">
         <v>55</v>
@@ -13394,7 +13359,7 @@
         <v>722</v>
       </c>
       <c r="C238" s="8">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D238" s="5" t="s">
         <v>42</v>
@@ -13406,7 +13371,7 @@
         <v>723</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H238" s="5" t="s">
         <v>55</v>
@@ -13420,7 +13385,7 @@
         <v>725</v>
       </c>
       <c r="C239" s="8">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D239" s="5" t="s">
         <v>42</v>
@@ -13432,7 +13397,7 @@
         <v>726</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H239" s="5" t="s">
         <v>55</v>
@@ -13446,7 +13411,7 @@
         <v>728</v>
       </c>
       <c r="C240" s="8">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>42</v>
@@ -13458,7 +13423,7 @@
         <v>729</v>
       </c>
       <c r="G240" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H240" s="5" t="s">
         <v>55</v>
@@ -13472,7 +13437,7 @@
         <v>731</v>
       </c>
       <c r="C241" s="8">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>42</v>
@@ -13484,7 +13449,7 @@
         <v>732</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H241" s="5" t="s">
         <v>55</v>
@@ -13498,7 +13463,7 @@
         <v>734</v>
       </c>
       <c r="C242" s="8">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D242" s="5" t="s">
         <v>42</v>
@@ -13510,7 +13475,7 @@
         <v>735</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H242" s="5" t="s">
         <v>55</v>
@@ -13524,7 +13489,7 @@
         <v>737</v>
       </c>
       <c r="C243" s="8">
-        <v>1</v>
+        <v>0.0015</v>
       </c>
       <c r="D243" s="5" t="s">
         <v>42</v>
@@ -13536,7 +13501,7 @@
         <v>738</v>
       </c>
       <c r="G243" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H243" s="5" t="s">
         <v>55</v>
@@ -13550,7 +13515,7 @@
         <v>740</v>
       </c>
       <c r="C244" s="8">
-        <v>0.0015</v>
+        <v>1.8</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>42</v>
@@ -13562,7 +13527,7 @@
         <v>741</v>
       </c>
       <c r="G244" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H244" s="5" t="s">
         <v>55</v>
@@ -13576,7 +13541,7 @@
         <v>743</v>
       </c>
       <c r="C245" s="8">
-        <v>1.8</v>
+        <v>45</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>42</v>
@@ -13588,7 +13553,7 @@
         <v>744</v>
       </c>
       <c r="G245" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H245" s="5" t="s">
         <v>55</v>
@@ -13602,7 +13567,7 @@
         <v>746</v>
       </c>
       <c r="C246" s="8">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>42</v>
@@ -13614,7 +13579,7 @@
         <v>747</v>
       </c>
       <c r="G246" s="5" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="H246" s="5" t="s">
         <v>55</v>
@@ -13627,8 +13592,8 @@
       <c r="B247" s="5" t="s">
         <v>749</v>
       </c>
-      <c r="C247" s="8">
-        <v>28</v>
+      <c r="C247" s="7">
+        <v>2</v>
       </c>
       <c r="D247" s="5" t="s">
         <v>42</v>
@@ -13640,33 +13605,33 @@
         <v>750</v>
       </c>
       <c r="G247" s="5" t="s">
-        <v>702</v>
+        <v>751</v>
       </c>
       <c r="H247" s="5" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="248" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A248" s="5" t="s">
+        <v>752</v>
+      </c>
+      <c r="B248" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="C248" s="7">
+        <v>4</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E248" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F248" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="G248" s="5" t="s">
         <v>751</v>
-      </c>
-      <c r="B248" s="5" t="s">
-        <v>752</v>
-      </c>
-      <c r="C248" s="7">
-        <v>2</v>
-      </c>
-      <c r="D248" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E248" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F248" s="5" t="s">
-        <v>753</v>
-      </c>
-      <c r="G248" s="5" t="s">
-        <v>754</v>
       </c>
       <c r="H248" s="5" t="s">
         <v>39</v>
@@ -13680,7 +13645,7 @@
         <v>756</v>
       </c>
       <c r="C249" s="7">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D249" s="5" t="s">
         <v>42</v>
@@ -13689,10 +13654,10 @@
         <v>3</v>
       </c>
       <c r="F249" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G249" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H249" s="5" t="s">
         <v>39</v>
@@ -13700,13 +13665,13 @@
     </row>
     <row r="250" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A250" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="B250" s="5" t="s">
         <v>758</v>
       </c>
-      <c r="B250" s="5" t="s">
-        <v>759</v>
-      </c>
       <c r="C250" s="7">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D250" s="5" t="s">
         <v>42</v>
@@ -13715,10 +13680,10 @@
         <v>3</v>
       </c>
       <c r="F250" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G250" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H250" s="5" t="s">
         <v>39</v>
@@ -13726,13 +13691,13 @@
     </row>
     <row r="251" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A251" s="5" t="s">
+        <v>759</v>
+      </c>
+      <c r="B251" s="5" t="s">
         <v>760</v>
       </c>
-      <c r="B251" s="5" t="s">
-        <v>761</v>
-      </c>
       <c r="C251" s="7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D251" s="5" t="s">
         <v>42</v>
@@ -13741,10 +13706,10 @@
         <v>3</v>
       </c>
       <c r="F251" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G251" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H251" s="5" t="s">
         <v>39</v>
@@ -13752,13 +13717,13 @@
     </row>
     <row r="252" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A252" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="B252" s="5" t="s">
         <v>762</v>
       </c>
-      <c r="B252" s="5" t="s">
-        <v>763</v>
-      </c>
       <c r="C252" s="7">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D252" s="5" t="s">
         <v>42</v>
@@ -13767,10 +13732,10 @@
         <v>3</v>
       </c>
       <c r="F252" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H252" s="5" t="s">
         <v>39</v>
@@ -13778,13 +13743,13 @@
     </row>
     <row r="253" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A253" s="5" t="s">
+        <v>763</v>
+      </c>
+      <c r="B253" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="B253" s="5" t="s">
-        <v>765</v>
-      </c>
       <c r="C253" s="7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D253" s="5" t="s">
         <v>42</v>
@@ -13793,10 +13758,10 @@
         <v>3</v>
       </c>
       <c r="F253" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G253" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H253" s="5" t="s">
         <v>39</v>
@@ -13804,13 +13769,13 @@
     </row>
     <row r="254" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A254" s="5" t="s">
+        <v>765</v>
+      </c>
+      <c r="B254" s="5" t="s">
         <v>766</v>
       </c>
-      <c r="B254" s="5" t="s">
-        <v>767</v>
-      </c>
       <c r="C254" s="7">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D254" s="5" t="s">
         <v>42</v>
@@ -13819,10 +13784,10 @@
         <v>3</v>
       </c>
       <c r="F254" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G254" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H254" s="5" t="s">
         <v>39</v>
@@ -13830,13 +13795,13 @@
     </row>
     <row r="255" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A255" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="B255" s="5" t="s">
         <v>768</v>
       </c>
-      <c r="B255" s="5" t="s">
-        <v>769</v>
-      </c>
       <c r="C255" s="7">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D255" s="5" t="s">
         <v>42</v>
@@ -13845,10 +13810,10 @@
         <v>3</v>
       </c>
       <c r="F255" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G255" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H255" s="5" t="s">
         <v>39</v>
@@ -13856,13 +13821,13 @@
     </row>
     <row r="256" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="B256" s="5" t="s">
         <v>770</v>
       </c>
-      <c r="B256" s="5" t="s">
-        <v>771</v>
-      </c>
       <c r="C256" s="7">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D256" s="5" t="s">
         <v>42</v>
@@ -13871,10 +13836,10 @@
         <v>3</v>
       </c>
       <c r="F256" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G256" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H256" s="5" t="s">
         <v>39</v>
@@ -13882,13 +13847,13 @@
     </row>
     <row r="257" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A257" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="B257" s="5" t="s">
         <v>772</v>
       </c>
-      <c r="B257" s="5" t="s">
-        <v>773</v>
-      </c>
       <c r="C257" s="7">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>42</v>
@@ -13897,10 +13862,10 @@
         <v>3</v>
       </c>
       <c r="F257" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H257" s="5" t="s">
         <v>39</v>
@@ -13908,13 +13873,13 @@
     </row>
     <row r="258" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A258" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="B258" s="5" t="s">
         <v>774</v>
       </c>
-      <c r="B258" s="5" t="s">
-        <v>775</v>
-      </c>
       <c r="C258" s="7">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>42</v>
@@ -13923,10 +13888,10 @@
         <v>3</v>
       </c>
       <c r="F258" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H258" s="5" t="s">
         <v>39</v>
@@ -13934,13 +13899,13 @@
     </row>
     <row r="259" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A259" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="B259" s="5" t="s">
         <v>776</v>
       </c>
-      <c r="B259" s="5" t="s">
-        <v>777</v>
-      </c>
       <c r="C259" s="7">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D259" s="5" t="s">
         <v>42</v>
@@ -13949,10 +13914,10 @@
         <v>3</v>
       </c>
       <c r="F259" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G259" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H259" s="5" t="s">
         <v>39</v>
@@ -13960,13 +13925,13 @@
     </row>
     <row r="260" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A260" s="5" t="s">
+        <v>777</v>
+      </c>
+      <c r="B260" s="5" t="s">
         <v>778</v>
       </c>
-      <c r="B260" s="5" t="s">
-        <v>779</v>
-      </c>
       <c r="C260" s="7">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="D260" s="5" t="s">
         <v>42</v>
@@ -13975,10 +13940,10 @@
         <v>3</v>
       </c>
       <c r="F260" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H260" s="5" t="s">
         <v>39</v>
@@ -13986,13 +13951,13 @@
     </row>
     <row r="261" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A261" s="5" t="s">
+        <v>779</v>
+      </c>
+      <c r="B261" s="5" t="s">
         <v>780</v>
       </c>
-      <c r="B261" s="5" t="s">
-        <v>781</v>
-      </c>
       <c r="C261" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D261" s="5" t="s">
         <v>42</v>
@@ -14001,10 +13966,10 @@
         <v>3</v>
       </c>
       <c r="F261" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G261" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H261" s="5" t="s">
         <v>39</v>
@@ -14012,13 +13977,13 @@
     </row>
     <row r="262" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A262" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="B262" s="5" t="s">
         <v>782</v>
       </c>
-      <c r="B262" s="5" t="s">
-        <v>783</v>
-      </c>
       <c r="C262" s="7">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>42</v>
@@ -14027,10 +13992,10 @@
         <v>3</v>
       </c>
       <c r="F262" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G262" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H262" s="5" t="s">
         <v>39</v>
@@ -14038,13 +14003,13 @@
     </row>
     <row r="263" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A263" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="B263" s="5" t="s">
         <v>784</v>
       </c>
-      <c r="B263" s="5" t="s">
-        <v>785</v>
-      </c>
       <c r="C263" s="7">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D263" s="5" t="s">
         <v>42</v>
@@ -14053,10 +14018,10 @@
         <v>3</v>
       </c>
       <c r="F263" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G263" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H263" s="5" t="s">
         <v>39</v>
@@ -14064,13 +14029,13 @@
     </row>
     <row r="264" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A264" s="5" t="s">
+        <v>785</v>
+      </c>
+      <c r="B264" s="5" t="s">
         <v>786</v>
       </c>
-      <c r="B264" s="5" t="s">
-        <v>787</v>
-      </c>
       <c r="C264" s="7">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D264" s="5" t="s">
         <v>42</v>
@@ -14079,10 +14044,10 @@
         <v>3</v>
       </c>
       <c r="F264" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G264" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H264" s="5" t="s">
         <v>39</v>
@@ -14090,13 +14055,13 @@
     </row>
     <row r="265" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A265" s="5" t="s">
+        <v>787</v>
+      </c>
+      <c r="B265" s="5" t="s">
         <v>788</v>
       </c>
-      <c r="B265" s="5" t="s">
-        <v>789</v>
-      </c>
       <c r="C265" s="7">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D265" s="5" t="s">
         <v>42</v>
@@ -14105,10 +14070,10 @@
         <v>3</v>
       </c>
       <c r="F265" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G265" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H265" s="5" t="s">
         <v>39</v>
@@ -14116,13 +14081,13 @@
     </row>
     <row r="266" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A266" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="B266" s="5" t="s">
         <v>790</v>
       </c>
-      <c r="B266" s="5" t="s">
-        <v>791</v>
-      </c>
       <c r="C266" s="7">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D266" s="5" t="s">
         <v>42</v>
@@ -14131,10 +14096,10 @@
         <v>3</v>
       </c>
       <c r="F266" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G266" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H266" s="5" t="s">
         <v>39</v>
@@ -14142,10 +14107,10 @@
     </row>
     <row r="267" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A267" s="5" t="s">
+        <v>791</v>
+      </c>
+      <c r="B267" s="5" t="s">
         <v>792</v>
-      </c>
-      <c r="B267" s="5" t="s">
-        <v>793</v>
       </c>
       <c r="C267" s="7">
         <v>35</v>
@@ -14157,10 +14122,10 @@
         <v>3</v>
       </c>
       <c r="F267" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H267" s="5" t="s">
         <v>39</v>
@@ -14168,13 +14133,13 @@
     </row>
     <row r="268" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A268" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="B268" s="5" t="s">
         <v>794</v>
       </c>
-      <c r="B268" s="5" t="s">
-        <v>795</v>
-      </c>
       <c r="C268" s="7">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D268" s="5" t="s">
         <v>42</v>
@@ -14183,10 +14148,10 @@
         <v>3</v>
       </c>
       <c r="F268" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G268" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H268" s="5" t="s">
         <v>39</v>
@@ -14194,13 +14159,13 @@
     </row>
     <row r="269" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A269" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="B269" s="5" t="s">
         <v>796</v>
       </c>
-      <c r="B269" s="5" t="s">
-        <v>797</v>
-      </c>
       <c r="C269" s="7">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D269" s="5" t="s">
         <v>42</v>
@@ -14209,10 +14174,10 @@
         <v>3</v>
       </c>
       <c r="F269" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G269" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H269" s="5" t="s">
         <v>39</v>
@@ -14220,13 +14185,13 @@
     </row>
     <row r="270" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A270" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="B270" s="5" t="s">
         <v>798</v>
       </c>
-      <c r="B270" s="5" t="s">
-        <v>799</v>
-      </c>
       <c r="C270" s="7">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D270" s="5" t="s">
         <v>42</v>
@@ -14235,10 +14200,10 @@
         <v>3</v>
       </c>
       <c r="F270" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G270" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H270" s="5" t="s">
         <v>39</v>
@@ -14246,13 +14211,13 @@
     </row>
     <row r="271" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A271" s="5" t="s">
+        <v>799</v>
+      </c>
+      <c r="B271" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="B271" s="5" t="s">
-        <v>801</v>
-      </c>
       <c r="C271" s="7">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D271" s="5" t="s">
         <v>42</v>
@@ -14261,10 +14226,10 @@
         <v>3</v>
       </c>
       <c r="F271" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G271" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H271" s="5" t="s">
         <v>39</v>
@@ -14272,13 +14237,13 @@
     </row>
     <row r="272" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A272" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="B272" s="5" t="s">
         <v>802</v>
       </c>
-      <c r="B272" s="5" t="s">
-        <v>803</v>
-      </c>
       <c r="C272" s="7">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="D272" s="5" t="s">
         <v>42</v>
@@ -14287,10 +14252,10 @@
         <v>3</v>
       </c>
       <c r="F272" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G272" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H272" s="5" t="s">
         <v>39</v>
@@ -14298,13 +14263,13 @@
     </row>
     <row r="273" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A273" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="B273" s="5" t="s">
         <v>804</v>
       </c>
-      <c r="B273" s="5" t="s">
-        <v>805</v>
-      </c>
       <c r="C273" s="7">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="D273" s="5" t="s">
         <v>42</v>
@@ -14313,10 +14278,10 @@
         <v>3</v>
       </c>
       <c r="F273" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G273" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H273" s="5" t="s">
         <v>39</v>
@@ -14324,13 +14289,13 @@
     </row>
     <row r="274" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A274" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="B274" s="5" t="s">
         <v>806</v>
       </c>
-      <c r="B274" s="5" t="s">
-        <v>807</v>
-      </c>
       <c r="C274" s="7">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D274" s="5" t="s">
         <v>42</v>
@@ -14339,10 +14304,10 @@
         <v>3</v>
       </c>
       <c r="F274" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G274" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H274" s="5" t="s">
         <v>39</v>
@@ -14350,13 +14315,13 @@
     </row>
     <row r="275" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A275" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="B275" s="5" t="s">
         <v>808</v>
       </c>
-      <c r="B275" s="5" t="s">
-        <v>809</v>
-      </c>
       <c r="C275" s="7">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D275" s="5" t="s">
         <v>42</v>
@@ -14365,10 +14330,10 @@
         <v>3</v>
       </c>
       <c r="F275" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G275" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H275" s="5" t="s">
         <v>39</v>
@@ -14376,13 +14341,13 @@
     </row>
     <row r="276" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="B276" s="5" t="s">
         <v>810</v>
       </c>
-      <c r="B276" s="5" t="s">
-        <v>811</v>
-      </c>
       <c r="C276" s="7">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>42</v>
@@ -14391,43 +14356,17 @@
         <v>3</v>
       </c>
       <c r="F276" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G276" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H276" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="277" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A277" s="5" t="s">
-        <v>812</v>
-      </c>
-      <c r="B277" s="5" t="s">
-        <v>813</v>
-      </c>
-      <c r="C277" s="7">
-        <v>5</v>
-      </c>
-      <c r="D277" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E277" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F277" s="5" t="s">
-        <v>757</v>
-      </c>
-      <c r="G277" s="5" t="s">
-        <v>754</v>
-      </c>
-      <c r="H277" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H277"/>
+  <autoFilter ref="A1:H276"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -14479,10 +14418,10 @@
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="C2" s="7">
         <v>2</v>
@@ -14494,10 +14433,10 @@
         <v>3</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>39</v>
@@ -14505,10 +14444,10 @@
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="C3" s="7">
         <v>4</v>
@@ -14520,10 +14459,10 @@
         <v>3</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>39</v>
@@ -14531,10 +14470,10 @@
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="C4" s="7">
         <v>12</v>
@@ -14546,10 +14485,10 @@
         <v>3</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>39</v>
@@ -14557,10 +14496,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="C5" s="7">
         <v>8</v>
@@ -14572,10 +14511,10 @@
         <v>3</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>39</v>
@@ -14583,10 +14522,10 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="C6" s="7">
         <v>3</v>
@@ -14598,10 +14537,10 @@
         <v>3</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>39</v>
@@ -14609,10 +14548,10 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="C7" s="7">
         <v>8</v>
@@ -14624,10 +14563,10 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>39</v>
@@ -14635,10 +14574,10 @@
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="C8" s="7">
         <v>12</v>
@@ -14650,10 +14589,10 @@
         <v>3</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>39</v>
@@ -14661,10 +14600,10 @@
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="C9" s="7">
         <v>24</v>
@@ -14676,10 +14615,10 @@
         <v>3</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>39</v>
@@ -14687,10 +14626,10 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="C10" s="7">
         <v>14</v>
@@ -14702,10 +14641,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>39</v>
@@ -14713,10 +14652,10 @@
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C11" s="7">
         <v>20</v>
@@ -14728,10 +14667,10 @@
         <v>3</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>39</v>
@@ -14739,10 +14678,10 @@
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="C12" s="7">
         <v>22</v>
@@ -14754,10 +14693,10 @@
         <v>3</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>39</v>
@@ -14765,10 +14704,10 @@
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C13" s="7">
         <v>30</v>
@@ -14780,10 +14719,10 @@
         <v>3</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>39</v>
@@ -14791,10 +14730,10 @@
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="C14" s="7">
         <v>40</v>
@@ -14806,10 +14745,10 @@
         <v>3</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>39</v>
@@ -14817,10 +14756,10 @@
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="C15" s="7">
         <v>5</v>
@@ -14832,10 +14771,10 @@
         <v>3</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>39</v>
@@ -14843,10 +14782,10 @@
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="C16" s="7">
         <v>8</v>
@@ -14858,10 +14797,10 @@
         <v>3</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>39</v>
@@ -14869,10 +14808,10 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="C17" s="7">
         <v>18</v>
@@ -14884,10 +14823,10 @@
         <v>3</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>39</v>
@@ -14895,10 +14834,10 @@
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="C18" s="7">
         <v>10</v>
@@ -14910,10 +14849,10 @@
         <v>3</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>39</v>
@@ -14921,10 +14860,10 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C19" s="7">
         <v>16</v>
@@ -14936,10 +14875,10 @@
         <v>3</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>39</v>
@@ -14947,10 +14886,10 @@
     </row>
     <row r="20" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="C20" s="7">
         <v>20</v>
@@ -14962,10 +14901,10 @@
         <v>3</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>39</v>
@@ -14973,10 +14912,10 @@
     </row>
     <row r="21" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C21" s="7">
         <v>35</v>
@@ -14988,10 +14927,10 @@
         <v>3</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H21" s="5" t="s">
         <v>39</v>
@@ -14999,10 +14938,10 @@
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="C22" s="7">
         <v>35</v>
@@ -15014,10 +14953,10 @@
         <v>3</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>39</v>
@@ -15025,10 +14964,10 @@
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="C23" s="7">
         <v>25</v>
@@ -15040,10 +14979,10 @@
         <v>3</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>39</v>
@@ -15051,10 +14990,10 @@
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C24" s="7">
         <v>32</v>
@@ -15066,10 +15005,10 @@
         <v>3</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>39</v>
@@ -15077,10 +15016,10 @@
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="C25" s="7">
         <v>38</v>
@@ -15092,10 +15031,10 @@
         <v>3</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>39</v>
@@ -15103,10 +15042,10 @@
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="C26" s="7">
         <v>34</v>
@@ -15118,10 +15057,10 @@
         <v>3</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>39</v>
@@ -15129,10 +15068,10 @@
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="C27" s="7">
         <v>60</v>
@@ -15144,10 +15083,10 @@
         <v>3</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>39</v>
@@ -15155,10 +15094,10 @@
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="C28" s="7">
         <v>8</v>
@@ -15170,10 +15109,10 @@
         <v>3</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>39</v>
@@ -15181,10 +15120,10 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="C29" s="7">
         <v>14</v>
@@ -15196,10 +15135,10 @@
         <v>3</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>39</v>
@@ -15207,10 +15146,10 @@
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="C30" s="7">
         <v>30</v>
@@ -15222,10 +15161,10 @@
         <v>3</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>39</v>
@@ -15233,10 +15172,10 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="C31" s="7">
         <v>5</v>
@@ -15248,10 +15187,10 @@
         <v>3</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>39</v>

</xml_diff>